<commit_message>
Hoàn thiện ~80%, tạm dừng để ôn thi, sẽ tiếp tục sau
</commit_message>
<xml_diff>
--- a/tools/sample_import.xlsx
+++ b/tools/sample_import.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="DauSach" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="BanSao" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="DocGia" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,6 +459,16 @@
           <t>tong_ban_sao</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>gia_tien</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>nha_xuat_ban</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -494,6 +505,14 @@
       <c r="H2" t="n">
         <v>2</v>
       </c>
+      <c r="I2" t="n">
+        <v>85000</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>NXB Giao Duc</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -529,6 +548,14 @@
       </c>
       <c r="H3" t="n">
         <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>120000</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>NXB Tre</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -629,4 +656,158 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ma_the</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ho</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ten</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>phai</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>trang_thai</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>so_dien_thoai</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>lop</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>ngay_sinh</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>loai_doc_gia</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>10001</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Nguyen</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>An</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0912345678</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>an.nv@gmail.com</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>12A1</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2006-05-15</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>10002</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Tran</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Binh</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0987654321</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>binh.tt@gmail.com</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>11B2</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2007-10-20</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>